<commit_message>
Replace Forman putty with Volma gypsum finishing putty.
Forman 20 kg is unavailable in Krasnodar; gypsum finishing putty is the in-store substitute for GKL joints and paint on an enclosed balcony.

Co-authored-by: Alena931 <Alena931@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/smeta-pervyy-balkon-krasnodar.xlsx
+++ b/smeta-pervyy-balkon-krasnodar.xlsx
@@ -839,7 +839,7 @@
     <row r="4">
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Дата составления: 12 октября 2026  •  Объект: первый балкон  •  Город: Краснодар</t>
+          <t>Дата составления: 13 октября 2026  •  Объект: первый балкон  •  Город: Краснодар</t>
         </is>
       </c>
     </row>
@@ -865,7 +865,7 @@
     </row>
     <row r="7" ht="32" customHeight="1">
       <c r="B7" s="10" t="n">
-        <v>21017</v>
+        <v>21030</v>
       </c>
       <c r="C7" s="11" t="n"/>
       <c r="D7" s="10" t="n">
@@ -873,7 +873,7 @@
       </c>
       <c r="E7" s="11" t="n"/>
       <c r="F7" s="10" t="n">
-        <v>44412</v>
+        <v>44425</v>
       </c>
       <c r="G7" s="11" t="n"/>
     </row>
@@ -1021,7 +1021,7 @@
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="1" fitToWidth="1"/>
   <headerFooter>
     <oddHeader>&amp;LПервый балкон — смета</oddHeader>
-    <oddFooter>&amp;LПервый балкон, Краснодар&amp;C12.10.2026&amp;R&amp;P из &amp;N</oddFooter>
+    <oddFooter>&amp;LПервый балкон, Краснодар&amp;C13.10.2026&amp;R&amp;P из &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -1585,12 +1585,12 @@
       </c>
       <c r="C14" s="38" t="inlineStr">
         <is>
-          <t>Шпатлёвка Forman гипсополимерная финишная 20 кг</t>
+          <t>Шпаклёвка гипсовая финишная Волма Финиш 20 кг</t>
         </is>
       </c>
       <c r="D14" s="37" t="inlineStr">
         <is>
-          <t>90639104</t>
+          <t>82034158</t>
         </is>
       </c>
       <c r="E14" s="37" t="inlineStr">
@@ -1602,10 +1602,10 @@
         <v>1</v>
       </c>
       <c r="G14" s="40" t="n">
-        <v>465</v>
+        <v>478</v>
       </c>
       <c r="H14" s="41" t="n">
-        <v>465</v>
+        <v>478</v>
       </c>
       <c r="I14" s="37" t="inlineStr">
         <is>
@@ -1614,7 +1614,7 @@
       </c>
       <c r="J14" s="38" t="inlineStr">
         <is>
-          <t>Сатентек в каталоге Лемана ПРО Краснодар не найден</t>
+          <t>Forman 20 кг в магазине нет. Гипсовая финишная — нормальная замена под покраску ГКЛ в сухом остеклённом балконе. Акция 478 ₽, без акции 582 ₽. Не для холодного балкона.</t>
         </is>
       </c>
       <c r="K14" s="42" t="inlineStr">
@@ -2185,7 +2185,7 @@
     <row r="28">
       <c r="A28" s="18" t="inlineStr">
         <is>
-          <t>Жёлтым отмечены замены: нет точной фасовки или бренда в каталоге Лемана ПРО Краснодар. Итог 21 017 ₽ — ориентир витрины, не счёт к оплате. Доставка в сумму материалов не входит.</t>
+          <t>Жёлтым отмечены замены: нет точной фасовки или бренда в каталоге Лемана ПРО Краснодар. Итог 21 030 ₽ — ориентир витрины, не счёт к оплате. Доставка в сумму материалов не входит.</t>
         </is>
       </c>
     </row>
@@ -2226,7 +2226,7 @@
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="1" fitToWidth="1"/>
   <headerFooter>
     <oddHeader>&amp;LМатериалы — Лемана ПРО, Краснодар</oddHeader>
-    <oddFooter>&amp;LПервый балкон, Краснодар&amp;C12.10.2026&amp;R&amp;P из &amp;N</oddFooter>
+    <oddFooter>&amp;LПервый балкон, Краснодар&amp;C13.10.2026&amp;R&amp;P из &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -3002,7 +3002,7 @@
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="1" fitToWidth="1"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;LПервый балкон, Краснодар&amp;C12.10.2026&amp;R&amp;P из &amp;N</oddFooter>
+    <oddFooter>&amp;LПервый балкон, Краснодар&amp;C13.10.2026&amp;R&amp;P из &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -3442,7 +3442,7 @@
     <row r="18">
       <c r="A18" s="58" t="inlineStr">
         <is>
-          <t>Итог. В оплату по этой смете входят только работы со листа «Работы», строки 1–10, на сумму 23 395 ₽. Всё перечисленное выше в 23 395 ₽ не входит. Материалы оплачиваются отдельно (~21 017 ₽ по листу «Материалы»).</t>
+          <t>Итог. В оплату по этой смете входят только работы со листа «Работы», строки 1–10, на сумму 23 395 ₽. Всё перечисленное выше в 23 395 ₽ не входит. Материалы оплачиваются отдельно (~21 030 ₽ по листу «Материалы»).</t>
         </is>
       </c>
       <c r="B18" s="59" t="n"/>
@@ -3477,7 +3477,7 @@
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="1" fitToWidth="1"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;LПервый балкон, Краснодар&amp;C12.10.2026&amp;R&amp;P из &amp;N</oddFooter>
+    <oddFooter>&amp;LПервый балкон, Краснодар&amp;C13.10.2026&amp;R&amp;P из &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>

</xml_diff>

<commit_message>
Replace composite mesh with in-store glass-fiber masonry mesh.
Same 0.5×2 m card, 50×50 mm cell and 2 mm rod; Krasnodar SKU 82471768 at 80 ₽.

Co-authored-by: Alena931 <Alena931@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/smeta-pervyy-balkon-krasnodar.xlsx
+++ b/smeta-pervyy-balkon-krasnodar.xlsx
@@ -865,7 +865,7 @@
     </row>
     <row r="7" ht="32" customHeight="1">
       <c r="B7" s="10" t="n">
-        <v>21030</v>
+        <v>20846</v>
       </c>
       <c r="C7" s="11" t="n"/>
       <c r="D7" s="10" t="n">
@@ -873,7 +873,7 @@
       </c>
       <c r="E7" s="11" t="n"/>
       <c r="F7" s="10" t="n">
-        <v>44425</v>
+        <v>44241</v>
       </c>
       <c r="G7" s="11" t="n"/>
     </row>
@@ -1820,49 +1820,49 @@
       </c>
     </row>
     <row r="19" ht="36" customHeight="1">
-      <c r="A19" s="24" t="n">
+      <c r="A19" s="37" t="n">
         <v>15</v>
       </c>
-      <c r="B19" s="25" t="inlineStr">
+      <c r="B19" s="38" t="inlineStr">
         <is>
           <t>Сетка композитная 50×50, 2 м × 50 см — 4 шт</t>
         </is>
       </c>
-      <c r="C19" s="25" t="inlineStr">
-        <is>
-          <t>Сетка композитная 50×50×2 мм, 0,5×2 м</t>
-        </is>
-      </c>
-      <c r="D19" s="24" t="inlineStr">
-        <is>
-          <t>86750000</t>
-        </is>
-      </c>
-      <c r="E19" s="24" t="inlineStr">
+      <c r="C19" s="38" t="inlineStr">
+        <is>
+          <t>Сетка клад. стеклопласт 50×50 мм Ø2 мм, 0,5×2 м</t>
+        </is>
+      </c>
+      <c r="D19" s="37" t="inlineStr">
+        <is>
+          <t>82471768</t>
+        </is>
+      </c>
+      <c r="E19" s="37" t="inlineStr">
         <is>
           <t>шт</t>
         </is>
       </c>
-      <c r="F19" s="26" t="n">
+      <c r="F19" s="39" t="n">
         <v>4</v>
       </c>
-      <c r="G19" s="27" t="n">
-        <v>126</v>
-      </c>
-      <c r="H19" s="28" t="n">
-        <v>504</v>
-      </c>
-      <c r="I19" s="24" t="inlineStr">
-        <is>
-          <t>как в списке</t>
-        </is>
-      </c>
-      <c r="J19" s="25" t="inlineStr">
-        <is>
-          <t>Размер полотна совпадает со списком</t>
-        </is>
-      </c>
-      <c r="K19" s="29" t="inlineStr">
+      <c r="G19" s="40" t="n">
+        <v>80</v>
+      </c>
+      <c r="H19" s="41" t="n">
+        <v>320</v>
+      </c>
+      <c r="I19" s="37" t="inlineStr">
+        <is>
+          <t>замена бренда</t>
+        </is>
+      </c>
+      <c r="J19" s="38" t="inlineStr">
+        <is>
+          <t>Композитной 86750000 в магазине нет. Та же карта 0,5×2 м, ячейка 50×50, пруток 2 мм — для стяжки на балконе подходит.</t>
+        </is>
+      </c>
+      <c r="K19" s="42" t="inlineStr">
         <is>
           <t>Открыть карточку</t>
         </is>
@@ -2185,7 +2185,7 @@
     <row r="28">
       <c r="A28" s="18" t="inlineStr">
         <is>
-          <t>Жёлтым отмечены замены: нет точной фасовки или бренда в каталоге Лемана ПРО Краснодар. Итог 21 030 ₽ — ориентир витрины, не счёт к оплате. Доставка в сумму материалов не входит.</t>
+          <t>Жёлтым отмечены замены: нет точной фасовки или бренда в каталоге Лемана ПРО Краснодар. Итог 20 846 ₽ — ориентир витрины, не счёт к оплате. Доставка в сумму материалов не входит.</t>
         </is>
       </c>
     </row>
@@ -3442,7 +3442,7 @@
     <row r="18">
       <c r="A18" s="58" t="inlineStr">
         <is>
-          <t>Итог. В оплату по этой смете входят только работы со листа «Работы», строки 1–10, на сумму 23 395 ₽. Всё перечисленное выше в 23 395 ₽ не входит. Материалы оплачиваются отдельно (~21 030 ₽ по листу «Материалы»).</t>
+          <t>Итог. В оплату по этой смете входят только работы со листа «Работы», строки 1–10, на сумму 23 395 ₽. Всё перечисленное выше в 23 395 ₽ не входит. Материалы оплачиваются отдельно (~20 846 ₽ по листу «Материалы»).</t>
         </is>
       </c>
       <c r="B18" s="59" t="n"/>

</xml_diff>

<commit_message>
Replace Stimul P-77 screed with Osnovit Pro 25 kg.
Fiber-reinforced cement screed, 20–200 mm, suitable over XPS on the balcony; Krasnodar SKU 82142242.

Co-authored-by: Alena931 <Alena931@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/smeta-pervyy-balkon-krasnodar.xlsx
+++ b/smeta-pervyy-balkon-krasnodar.xlsx
@@ -865,7 +865,7 @@
     </row>
     <row r="7" ht="32" customHeight="1">
       <c r="B7" s="10" t="n">
-        <v>20846</v>
+        <v>21086</v>
       </c>
       <c r="C7" s="11" t="n"/>
       <c r="D7" s="10" t="n">
@@ -873,7 +873,7 @@
       </c>
       <c r="E7" s="11" t="n"/>
       <c r="F7" s="10" t="n">
-        <v>44241</v>
+        <v>44481</v>
       </c>
       <c r="G7" s="11" t="n"/>
     </row>
@@ -1879,12 +1879,12 @@
       </c>
       <c r="C20" s="38" t="inlineStr">
         <is>
-          <t>Стяжка пола Стимул П-77, 25 кг</t>
+          <t>Стяжка пола Основит Pro 25 кг</t>
         </is>
       </c>
       <c r="D20" s="37" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>82142242</t>
         </is>
       </c>
       <c r="E20" s="37" t="inlineStr">
@@ -1896,19 +1896,19 @@
         <v>8</v>
       </c>
       <c r="G20" s="40" t="n">
-        <v>300</v>
+        <v>330</v>
       </c>
       <c r="H20" s="41" t="n">
-        <v>2400</v>
+        <v>2640</v>
       </c>
       <c r="I20" s="37" t="inlineStr">
         <is>
-          <t>замена фасовки</t>
+          <t>замена бренда</t>
         </is>
       </c>
       <c r="J20" s="38" t="inlineStr">
         <is>
-          <t>Мешков 30 кг в каталоге не найдено, взяты 25 кг × 8 шт как в списке</t>
+          <t>Стимул П-77 в магазине нет. Цементная с фиброй, слой 20–200 мм — на Пеноплэкс подходит. 8×25 кг ≈ 3 см на 3,5 м².</t>
         </is>
       </c>
       <c r="K20" s="42" t="inlineStr">
@@ -2185,7 +2185,7 @@
     <row r="28">
       <c r="A28" s="18" t="inlineStr">
         <is>
-          <t>Жёлтым отмечены замены: нет точной фасовки или бренда в каталоге Лемана ПРО Краснодар. Итог 20 846 ₽ — ориентир витрины, не счёт к оплате. Доставка в сумму материалов не входит.</t>
+          <t>Жёлтым отмечены замены: нет точной фасовки или бренда в каталоге Лемана ПРО Краснодар. Итог 21 086 ₽ — ориентир витрины, не счёт к оплате. Доставка в сумму материалов не входит.</t>
         </is>
       </c>
     </row>
@@ -3442,7 +3442,7 @@
     <row r="18">
       <c r="A18" s="58" t="inlineStr">
         <is>
-          <t>Итог. В оплату по этой смете входят только работы со листа «Работы», строки 1–10, на сумму 23 395 ₽. Всё перечисленное выше в 23 395 ₽ не входит. Материалы оплачиваются отдельно (~20 846 ₽ по листу «Материалы»).</t>
+          <t>Итог. В оплату по этой смете входят только работы со листа «Работы», строки 1–10, на сумму 23 395 ₽. Всё перечисленное выше в 23 395 ₽ не входит. Материалы оплачиваются отдельно (~21 086 ₽ по листу «Материалы»).</t>
         </is>
       </c>
       <c r="B18" s="59" t="n"/>

</xml_diff>

<commit_message>
Pin 10 mm galvanized beacon profile SKU 89474349.
22 mm is the flange width; working height stays 10 mm, same as the original plastic beacon.

Co-authored-by: Alena931 <Alena931@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/smeta-pervyy-balkon-krasnodar.xlsx
+++ b/smeta-pervyy-balkon-krasnodar.xlsx
@@ -1928,12 +1928,12 @@
       </c>
       <c r="C21" s="38" t="inlineStr">
         <is>
-          <t>Профиль маячковый (ПМ) Премиум 10×3000 мм</t>
+          <t>Профиль маячковый (ПМ) Премиум 10 мм оцинк. 22×3000 мм</t>
         </is>
       </c>
       <c r="D21" s="37" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>89474349</t>
         </is>
       </c>
       <c r="E21" s="37" t="inlineStr">
@@ -1957,7 +1957,7 @@
       </c>
       <c r="J21" s="38" t="inlineStr">
         <is>
-          <t>Пластиковый маяк 10 мм в выдаче не найден, взят маяк 10 мм / 3 м</t>
+          <t>22 мм — ширина полки, 10 мм — высота (то что нужно). Пластикового нет, оцинкованный 10 мм / 3 м ставится на раствор до слоя ~3 см.</t>
         </is>
       </c>
       <c r="K21" s="42" t="inlineStr">

</xml_diff>

<commit_message>
Replace long-lead Absolute paint with in-store Luxens 10 L.
Washable kitchen-and-bath matte white, article 81963491, typical Lemana PRO shelf stock.

Co-authored-by: Alena931 <Alena931@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/smeta-pervyy-balkon-krasnodar.xlsx
+++ b/smeta-pervyy-balkon-krasnodar.xlsx
@@ -865,7 +865,7 @@
     </row>
     <row r="7" ht="32" customHeight="1">
       <c r="B7" s="10" t="n">
-        <v>21086</v>
+        <v>20708</v>
       </c>
       <c r="C7" s="11" t="n"/>
       <c r="D7" s="10" t="n">
@@ -873,7 +873,7 @@
       </c>
       <c r="E7" s="11" t="n"/>
       <c r="F7" s="10" t="n">
-        <v>44481</v>
+        <v>44103</v>
       </c>
       <c r="G7" s="11" t="n"/>
     </row>
@@ -1634,12 +1634,12 @@
       </c>
       <c r="C15" s="38" t="inlineStr">
         <is>
-          <t>Краска Absolute Professional UniFarbe матовая белая 10 л</t>
+          <t>Краска для стен кухни и ванной Luxens матовая белая база А 10 л</t>
         </is>
       </c>
       <c r="D15" s="37" t="inlineStr">
         <is>
-          <t>92757425</t>
+          <t>81963491</t>
         </is>
       </c>
       <c r="E15" s="37" t="inlineStr">
@@ -1651,19 +1651,19 @@
         <v>1</v>
       </c>
       <c r="G15" s="40" t="n">
-        <v>3950</v>
+        <v>3572</v>
       </c>
       <c r="H15" s="41" t="n">
-        <v>3950</v>
+        <v>3572</v>
       </c>
       <c r="I15" s="37" t="inlineStr">
         <is>
-          <t>замена фасовки</t>
+          <t>замена бренда</t>
         </is>
       </c>
       <c r="J15" s="38" t="inlineStr">
         <is>
-          <t>Банки ровно 7 л нет, взята белая интерьерная 10 л</t>
+          <t>У Absolute долгая доставка. Luxens — свой бренд Лемана, обычно на полке. Моющаяся, ГКЛ, 10 л. Не брать базу С (только под колеровку).</t>
         </is>
       </c>
       <c r="K15" s="42" t="inlineStr">
@@ -2185,7 +2185,7 @@
     <row r="28">
       <c r="A28" s="18" t="inlineStr">
         <is>
-          <t>Жёлтым отмечены замены: нет точной фасовки или бренда в каталоге Лемана ПРО Краснодар. Итог 21 086 ₽ — ориентир витрины, не счёт к оплате. Доставка в сумму материалов не входит.</t>
+          <t>Жёлтым отмечены замены: нет точной фасовки или бренда в каталоге Лемана ПРО Краснодар. Итог 20 708 ₽ — ориентир витрины, не счёт к оплате. Доставка в сумму материалов не входит.</t>
         </is>
       </c>
     </row>
@@ -3442,7 +3442,7 @@
     <row r="18">
       <c r="A18" s="58" t="inlineStr">
         <is>
-          <t>Итог. В оплату по этой смете входят только работы со листа «Работы», строки 1–10, на сумму 23 395 ₽. Всё перечисленное выше в 23 395 ₽ не входит. Материалы оплачиваются отдельно (~21 086 ₽ по листу «Материалы»).</t>
+          <t>Итог. В оплату по этой смете входят только работы со листа «Работы», строки 1–10, на сумму 23 395 ₽. Всё перечисленное выше в 23 395 ₽ не входит. Материалы оплачиваются отдельно (~20 708 ₽ по листу «Материалы»).</t>
         </is>
       </c>
       <c r="B18" s="59" t="n"/>

</xml_diff>

<commit_message>
Recalc labor for both balconies without windowsills.
Same Krasnodar 2026 rates on each balcony from the materials lists:
9 m² of frame/GKL/wool/finish and 3.5 m² of floor, no sill install.
22 495 ₽ per balcony, 44 990 ₽ combined.

Co-authored-by: Alena931 <Alena931@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/smeta-pervyy-balkon-krasnodar.xlsx
+++ b/smeta-pervyy-balkon-krasnodar.xlsx
@@ -16,7 +16,6 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Сводка'!$1:$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Материалы'!$A$4:$K$26</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Материалы'!$1:$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Работы'!$A$4:$H$14</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Работы'!$1:$4</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'Не входит в работы'!$1:$4</definedName>
   </definedNames>
@@ -167,7 +166,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="13">
+  <fills count="14">
     <fill>
       <patternFill/>
     </fill>
@@ -222,6 +221,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFF4D6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F5F5F5"/>
       </patternFill>
     </fill>
     <fill>
@@ -300,7 +304,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="60">
+  <cellXfs count="69">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -404,6 +408,24 @@
     <xf numFmtId="0" fontId="17" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="15" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="15" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="18" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
@@ -411,16 +433,23 @@
     <xf numFmtId="164" fontId="8" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="167" fontId="15" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="167" fontId="15" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="18" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="19" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -825,55 +854,55 @@
     <row r="2" ht="28" customHeight="1">
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>СМЕТА НА ПЕРВЫЙ БАЛКОН</t>
+          <t>СМЕТА РАБОТ НА ДВА БАЛКОНА</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Материалы — Лемана ПРО, Краснодар  •  Работы — средние расценки Краснодара</t>
+          <t>Работы — средние расценки Краснодара  •  Подоконники не входят  •  Материалы — отдельный лист и корзина</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Дата составления: 13 октября 2026  •  Объект: первый балкон  •  Город: Краснодар</t>
+          <t>Дата составления: 13 октября 2026  •  Объект: два балкона  •  Город: Краснодар</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Материалы</t>
+          <t>Работы, балкон 1</t>
         </is>
       </c>
       <c r="C6" s="5" t="n"/>
       <c r="D6" s="6" t="inlineStr">
         <is>
-          <t>Работы</t>
+          <t>Работы, балкон 2</t>
         </is>
       </c>
       <c r="E6" s="7" t="n"/>
       <c r="F6" s="8" t="inlineStr">
         <is>
-          <t>Итого под ключ</t>
+          <t>Работы, оба</t>
         </is>
       </c>
       <c r="G6" s="9" t="n"/>
     </row>
     <row r="7" ht="32" customHeight="1">
       <c r="B7" s="10" t="n">
-        <v>20708</v>
+        <v>22495</v>
       </c>
       <c r="C7" s="11" t="n"/>
       <c r="D7" s="10" t="n">
-        <v>23395</v>
+        <v>22495</v>
       </c>
       <c r="E7" s="11" t="n"/>
       <c r="F7" s="10" t="n">
-        <v>44103</v>
+        <v>44990</v>
       </c>
       <c r="G7" s="11" t="n"/>
     </row>
@@ -887,10 +916,10 @@
     <row r="10" ht="20" customHeight="1">
       <c r="B10" s="13" t="inlineStr">
         <is>
-          <t>Объёмы работ посчитаны по списку материалов заказчика:
-• 3 листа ГКЛ 2500×1200 мм = 9,0 м² стен/потолка (каркас, минвата, шпаклёвка, грунтовка, покраска);
-• 5 листов Пеноплэкс 50 мм ≈ 3,5 м² пола (утепление, сетка, стяжка);
-• подоконник 1,5 м + заглушка + пена.</t>
+          <t>Объёмы по спискам материалов, без замера:
+• каждый балкон: 3 листа ГКЛ = 9,0 м² стен/потолка (каркас, минвата, шпаклёвка, грунт, покраска);
+• каждый балкон: 5 листов Пеноплэкс 50 мм ≈ 3,5 м² пола (утепление, сетка, стяжка);
+• подоконники не делаются. Шпаклёвка/грунт/краска в корзине общие, работа — на каждом балконе.</t>
         </is>
       </c>
     </row>
@@ -1020,8 +1049,8 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="1" fitToWidth="1"/>
   <headerFooter>
-    <oddHeader>&amp;LПервый балкон — смета</oddHeader>
-    <oddFooter>&amp;LПервый балкон, Краснодар&amp;C13.10.2026&amp;R&amp;P из &amp;N</oddFooter>
+    <oddHeader>&amp;LДва балкона — смета работ</oddHeader>
+    <oddFooter>&amp;LДва балкона, Краснодар&amp;C13.10.2026&amp;R&amp;P из &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -1055,7 +1084,7 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="20" t="inlineStr">
         <is>
-          <t>СМЕТА МАТЕРИАЛОВ  •  Лемана ПРО, Краснодар  •  первый балкон</t>
+          <t>СМЕТА МАТЕРИАЛОВ  •  Лемана ПРО, Краснодар  •  ориентир по балкону 1; корзина — на оба</t>
         </is>
       </c>
       <c r="B1" s="21" t="n"/>
@@ -1967,98 +1996,98 @@
       </c>
     </row>
     <row r="22" ht="36" customHeight="1">
-      <c r="A22" s="30" t="n">
+      <c r="A22" s="43" t="n">
         <v>18</v>
       </c>
-      <c r="B22" s="31" t="inlineStr">
+      <c r="B22" s="44" t="inlineStr">
         <is>
           <t>Подоконник 1,5 м × 20 см — 1 шт</t>
         </is>
       </c>
-      <c r="C22" s="31" t="inlineStr">
+      <c r="C22" s="44" t="inlineStr">
         <is>
           <t>Подоконник ПВХ 1500×200 мм, белый</t>
         </is>
       </c>
-      <c r="D22" s="30" t="inlineStr">
+      <c r="D22" s="43" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E22" s="30" t="inlineStr">
+      <c r="E22" s="43" t="inlineStr">
         <is>
           <t>шт</t>
         </is>
       </c>
-      <c r="F22" s="32" t="n">
-        <v>1</v>
-      </c>
-      <c r="G22" s="33" t="n">
+      <c r="F22" s="45" t="n">
+        <v>0</v>
+      </c>
+      <c r="G22" s="46" t="n">
         <v>360</v>
       </c>
-      <c r="H22" s="34" t="n">
-        <v>360</v>
-      </c>
-      <c r="I22" s="30" t="inlineStr">
-        <is>
-          <t>как в списке</t>
-        </is>
-      </c>
-      <c r="J22" s="31" t="inlineStr">
-        <is>
-          <t>Белый ПВХ 1500×200 мм</t>
-        </is>
-      </c>
-      <c r="K22" s="35" t="inlineStr">
+      <c r="H22" s="47" t="n">
+        <v>0</v>
+      </c>
+      <c r="I22" s="43" t="inlineStr">
+        <is>
+          <t>не делается</t>
+        </is>
+      </c>
+      <c r="J22" s="44" t="inlineStr">
+        <is>
+          <t>Заказчик подтвердил: подоконник не покупать и не монтировать</t>
+        </is>
+      </c>
+      <c r="K22" s="48" t="inlineStr">
         <is>
           <t>Открыть карточку</t>
         </is>
       </c>
     </row>
     <row r="23" ht="36" customHeight="1">
-      <c r="A23" s="24" t="n">
+      <c r="A23" s="43" t="n">
         <v>19</v>
       </c>
-      <c r="B23" s="25" t="inlineStr">
+      <c r="B23" s="44" t="inlineStr">
         <is>
           <t>Заглушка подоконника — 1 шт</t>
         </is>
       </c>
-      <c r="C23" s="25" t="inlineStr">
+      <c r="C23" s="44" t="inlineStr">
         <is>
           <t>Заглушка для подоконника ПВХ двухсторонняя</t>
         </is>
       </c>
-      <c r="D23" s="24" t="inlineStr">
+      <c r="D23" s="43" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E23" s="24" t="inlineStr">
+      <c r="E23" s="43" t="inlineStr">
         <is>
           <t>шт</t>
         </is>
       </c>
-      <c r="F23" s="26" t="n">
-        <v>1</v>
-      </c>
-      <c r="G23" s="27" t="n">
+      <c r="F23" s="45" t="n">
+        <v>0</v>
+      </c>
+      <c r="G23" s="46" t="n">
         <v>20</v>
       </c>
-      <c r="H23" s="28" t="n">
-        <v>20</v>
-      </c>
-      <c r="I23" s="24" t="inlineStr">
-        <is>
-          <t>как в списке</t>
-        </is>
-      </c>
-      <c r="J23" s="25" t="inlineStr">
-        <is>
-          <t>Торцевая заглушка, цвет уточнить к подоконнику</t>
-        </is>
-      </c>
-      <c r="K23" s="29" t="inlineStr">
+      <c r="H23" s="47" t="n">
+        <v>0</v>
+      </c>
+      <c r="I23" s="43" t="inlineStr">
+        <is>
+          <t>не делается</t>
+        </is>
+      </c>
+      <c r="J23" s="44" t="inlineStr">
+        <is>
+          <t>Заглушка к подоконнику не нужна</t>
+        </is>
+      </c>
+      <c r="K23" s="48" t="inlineStr">
         <is>
           <t>Открыть карточку</t>
         </is>
@@ -2163,18 +2192,18 @@
       </c>
     </row>
     <row r="26" ht="24" customHeight="1">
-      <c r="A26" s="43" t="inlineStr">
+      <c r="A26" s="49" t="inlineStr">
         <is>
           <t>ИТОГО МАТЕРИАЛЫ</t>
         </is>
       </c>
-      <c r="B26" s="44" t="n"/>
-      <c r="C26" s="44" t="n"/>
-      <c r="D26" s="44" t="n"/>
-      <c r="E26" s="44" t="n"/>
-      <c r="F26" s="44" t="n"/>
-      <c r="G26" s="44" t="n"/>
-      <c r="H26" s="45">
+      <c r="B26" s="50" t="n"/>
+      <c r="C26" s="50" t="n"/>
+      <c r="D26" s="50" t="n"/>
+      <c r="E26" s="50" t="n"/>
+      <c r="F26" s="50" t="n"/>
+      <c r="G26" s="50" t="n"/>
+      <c r="H26" s="51">
         <f>SUM(H5:H25)</f>
         <v/>
       </c>
@@ -2185,7 +2214,7 @@
     <row r="28">
       <c r="A28" s="18" t="inlineStr">
         <is>
-          <t>Жёлтым отмечены замены: нет точной фасовки или бренда в каталоге Лемана ПРО Краснодар. Итог 20 708 ₽ — ориентир витрины, не счёт к оплате. Доставка в сумму материалов не входит.</t>
+          <t>Жёлтым отмечены замены: нет точной фасовки или бренда в каталоге Лемана ПРО Краснодар. Подоконник и заглушка исключены (0 ₽). Итог листа — ориентир витрины по балкону 1, не счёт к оплате. Доставка не входит. Корзина на оба балкона — отдельно.</t>
         </is>
       </c>
     </row>
@@ -2226,7 +2255,7 @@
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="1" fitToWidth="1"/>
   <headerFooter>
     <oddHeader>&amp;LМатериалы — Лемана ПРО, Краснодар</oddHeader>
-    <oddFooter>&amp;LПервый балкон, Краснодар&amp;C13.10.2026&amp;R&amp;P из &amp;N</oddFooter>
+    <oddFooter>&amp;LДва балкона, Краснодар&amp;C13.10.2026&amp;R&amp;P из &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -2241,7 +2270,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H31"/>
+  <dimension ref="A1:H46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2257,7 +2286,7 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="20" t="inlineStr">
         <is>
-          <t>СМЕТА РАБОТ  •  средние цены Краснодара  •  первый балкон</t>
+          <t>СМЕТА РАБОТ  •  средние цены Краснодара  •  два балкона</t>
         </is>
       </c>
       <c r="B1" s="21" t="n"/>
@@ -2271,738 +2300,1117 @@
     <row r="2">
       <c r="A2" s="22" t="inlineStr">
         <is>
-          <t>Только работа, без стоимости материалов. Ставки — среднее по открытым прайсам Краснодара на 2026 год (не минимальная цена с Авито).</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="23" t="inlineStr">
+          <t>Только работа, без материалов. Ставки — среднее по открытым прайсам Краснодара на 2026 год. Подоконники не входят. Шпаклёвка, грунт и покраска — на каждом балконе, материалы в корзине общие.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="22" customHeight="1">
+      <c r="A4" s="52" t="inlineStr">
+        <is>
+          <t>БАЛКОН 1</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="n"/>
+      <c r="C4" s="7" t="n"/>
+      <c r="D4" s="7" t="n"/>
+      <c r="E4" s="7" t="n"/>
+      <c r="F4" s="7" t="n"/>
+      <c r="G4" s="7" t="n"/>
+      <c r="H4" s="7" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="23" t="inlineStr">
         <is>
           <t>№</t>
         </is>
       </c>
-      <c r="B4" s="23" t="inlineStr">
+      <c r="B5" s="23" t="inlineStr">
         <is>
           <t>Вид работ</t>
         </is>
       </c>
-      <c r="C4" s="23" t="inlineStr">
+      <c r="C5" s="23" t="inlineStr">
         <is>
           <t>Обоснование объёма</t>
         </is>
       </c>
-      <c r="D4" s="23" t="inlineStr">
+      <c r="D5" s="23" t="inlineStr">
         <is>
           <t>Ед.</t>
         </is>
       </c>
-      <c r="E4" s="23" t="inlineStr">
+      <c r="E5" s="23" t="inlineStr">
         <is>
           <t>Кол-во</t>
         </is>
       </c>
-      <c r="F4" s="23" t="inlineStr">
+      <c r="F5" s="23" t="inlineStr">
         <is>
           <t>Ставка, ₽</t>
         </is>
       </c>
-      <c r="G4" s="23" t="inlineStr">
+      <c r="G5" s="23" t="inlineStr">
         <is>
           <t>Сумма, ₽</t>
         </is>
       </c>
-      <c r="H4" s="23" t="inlineStr">
+      <c r="H5" s="23" t="inlineStr">
         <is>
           <t>Примечание</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="38" customHeight="1">
-      <c r="A5" s="24" t="n">
+    <row r="6" ht="38" customHeight="1">
+      <c r="A6" s="24" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="25" t="inlineStr">
+      <c r="B6" s="25" t="inlineStr">
         <is>
           <t>Каркас из ППН 27/28 и ПП 60/27, жёсткие подвесы, обшивка ГКЛ 12,5 мм</t>
         </is>
       </c>
-      <c r="C5" s="25" t="inlineStr">
+      <c r="C6" s="25" t="inlineStr">
         <is>
           <t>3 листа ГКЛ × 3 м² = 9,0 м²</t>
         </is>
       </c>
-      <c r="D5" s="24" t="inlineStr">
+      <c r="D6" s="24" t="inlineStr">
         <is>
           <t>м²</t>
         </is>
       </c>
-      <c r="E5" s="46" t="n">
+      <c r="E6" s="53" t="n">
         <v>9</v>
       </c>
-      <c r="F5" s="27" t="n">
+      <c r="F6" s="27" t="n">
         <v>650</v>
       </c>
-      <c r="G5" s="28" t="n">
+      <c r="G6" s="28" t="n">
         <v>5850</v>
       </c>
-      <c r="H5" s="25" t="inlineStr">
+      <c r="H6" s="25" t="inlineStr">
         <is>
           <t>Среднее 430–850 ₽/м² по прайсам Краснодара</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="38" customHeight="1">
-      <c r="A6" s="30" t="n">
+    <row r="7" ht="38" customHeight="1">
+      <c r="A7" s="30" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="31" t="inlineStr">
+      <c r="B7" s="31" t="inlineStr">
         <is>
           <t>Утепление каркаса минеральной ватой 50 мм</t>
         </is>
       </c>
-      <c r="C6" s="31" t="inlineStr">
+      <c r="C7" s="31" t="inlineStr">
         <is>
           <t>Площадь обшивки ГКЛ 9,0 м²</t>
         </is>
       </c>
-      <c r="D6" s="30" t="inlineStr">
+      <c r="D7" s="30" t="inlineStr">
         <is>
           <t>м²</t>
         </is>
       </c>
-      <c r="E6" s="47" t="n">
+      <c r="E7" s="54" t="n">
         <v>9</v>
       </c>
-      <c r="F6" s="33" t="n">
+      <c r="F7" s="33" t="n">
         <v>450</v>
       </c>
-      <c r="G6" s="34" t="n">
+      <c r="G7" s="34" t="n">
         <v>4050</v>
       </c>
-      <c r="H6" s="31" t="inlineStr">
+      <c r="H7" s="31" t="inlineStr">
         <is>
           <t>Среднее 400–700 ₽/м², работа без материала</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="38" customHeight="1">
-      <c r="A7" s="24" t="n">
+    <row r="8" ht="38" customHeight="1">
+      <c r="A8" s="24" t="n">
         <v>3</v>
       </c>
-      <c r="B7" s="25" t="inlineStr">
+      <c r="B8" s="25" t="inlineStr">
         <is>
           <t>Заделка швов бумажной лентой, шпаклёвка под покраску</t>
         </is>
       </c>
-      <c r="C7" s="25" t="inlineStr">
+      <c r="C8" s="25" t="inlineStr">
         <is>
           <t>Площадь ГКЛ 9,0 м²</t>
         </is>
       </c>
-      <c r="D7" s="24" t="inlineStr">
+      <c r="D8" s="24" t="inlineStr">
         <is>
           <t>м²</t>
         </is>
       </c>
-      <c r="E7" s="46" t="n">
+      <c r="E8" s="53" t="n">
         <v>9</v>
       </c>
-      <c r="F7" s="27" t="n">
+      <c r="F8" s="27" t="n">
         <v>380</v>
       </c>
-      <c r="G7" s="28" t="n">
+      <c r="G8" s="28" t="n">
         <v>3420</v>
       </c>
-      <c r="H7" s="25" t="inlineStr">
+      <c r="H8" s="25" t="inlineStr">
         <is>
           <t>Комплекс под покраску, среднее 320–400 ₽/м²</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="38" customHeight="1">
-      <c r="A8" s="30" t="n">
+    <row r="9" ht="38" customHeight="1">
+      <c r="A9" s="30" t="n">
         <v>4</v>
       </c>
-      <c r="B8" s="31" t="inlineStr">
+      <c r="B9" s="31" t="inlineStr">
         <is>
           <t>Грунтовка интерьерная, 2 раза</t>
         </is>
       </c>
-      <c r="C8" s="31" t="inlineStr">
+      <c r="C9" s="31" t="inlineStr">
         <is>
           <t>Площадь ГКЛ 9,0 м²</t>
         </is>
       </c>
-      <c r="D8" s="30" t="inlineStr">
+      <c r="D9" s="30" t="inlineStr">
         <is>
           <t>м²</t>
         </is>
       </c>
-      <c r="E8" s="47" t="n">
+      <c r="E9" s="54" t="n">
         <v>9</v>
       </c>
-      <c r="F8" s="33" t="n">
+      <c r="F9" s="33" t="n">
         <v>120</v>
       </c>
-      <c r="G8" s="34" t="n">
+      <c r="G9" s="34" t="n">
         <v>1080</v>
       </c>
-      <c r="H8" s="31" t="inlineStr">
+      <c r="H9" s="31" t="inlineStr">
         <is>
           <t>По 60 ₽/м² за проход: до шпаклёвки и перед краской</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="38" customHeight="1">
-      <c r="A9" s="24" t="n">
+    <row r="10" ht="38" customHeight="1">
+      <c r="A10" s="24" t="n">
         <v>5</v>
       </c>
-      <c r="B9" s="25" t="inlineStr">
+      <c r="B10" s="25" t="inlineStr">
         <is>
           <t>Покраска стен/потолка, 2 слоя</t>
         </is>
       </c>
-      <c r="C9" s="25" t="inlineStr">
+      <c r="C10" s="25" t="inlineStr">
         <is>
           <t>Площадь ГКЛ 9,0 м²</t>
         </is>
       </c>
-      <c r="D9" s="24" t="inlineStr">
+      <c r="D10" s="24" t="inlineStr">
         <is>
           <t>м²</t>
         </is>
       </c>
-      <c r="E9" s="46" t="n">
+      <c r="E10" s="53" t="n">
         <v>9</v>
       </c>
-      <c r="F9" s="27" t="n">
+      <c r="F10" s="27" t="n">
         <v>260</v>
       </c>
-      <c r="G9" s="28" t="n">
+      <c r="G10" s="28" t="n">
         <v>2340</v>
       </c>
-      <c r="H9" s="25" t="inlineStr">
+      <c r="H10" s="25" t="inlineStr">
         <is>
           <t>Среднее 220–300 ₽/м² за 2 слоя</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="38" customHeight="1">
-      <c r="A10" s="30" t="n">
+    <row r="11" ht="38" customHeight="1">
+      <c r="A11" s="30" t="n">
         <v>6</v>
       </c>
-      <c r="B10" s="31" t="inlineStr">
+      <c r="B11" s="31" t="inlineStr">
         <is>
           <t>Утепление пола Пеноплэксом 50 мм, крепление грибами</t>
         </is>
       </c>
-      <c r="C10" s="31" t="inlineStr">
+      <c r="C11" s="31" t="inlineStr">
         <is>
           <t>5 листов × 0,69 м² ≈ 3,5 м²</t>
         </is>
       </c>
-      <c r="D10" s="30" t="inlineStr">
+      <c r="D11" s="30" t="inlineStr">
         <is>
           <t>м²</t>
         </is>
       </c>
-      <c r="E10" s="47" t="n">
+      <c r="E11" s="54" t="n">
         <v>3.5</v>
       </c>
-      <c r="F10" s="33" t="n">
+      <c r="F11" s="33" t="n">
         <v>400</v>
       </c>
-      <c r="G10" s="34" t="n">
+      <c r="G11" s="34" t="n">
         <v>1400</v>
       </c>
-      <c r="H10" s="31" t="inlineStr">
+      <c r="H11" s="31" t="inlineStr">
         <is>
           <t>Работа по полу, без материала</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="38" customHeight="1">
-      <c r="A11" s="24" t="n">
+    <row r="12" ht="38" customHeight="1">
+      <c r="A12" s="24" t="n">
         <v>7</v>
       </c>
-      <c r="B11" s="25" t="inlineStr">
+      <c r="B12" s="25" t="inlineStr">
         <is>
           <t>Армирование стяжки композитной сеткой 50×50</t>
         </is>
       </c>
-      <c r="C11" s="25" t="inlineStr">
+      <c r="C12" s="25" t="inlineStr">
         <is>
           <t>Площадь пола ≈ 3,5 м²</t>
         </is>
       </c>
-      <c r="D11" s="24" t="inlineStr">
+      <c r="D12" s="24" t="inlineStr">
         <is>
           <t>м²</t>
         </is>
       </c>
-      <c r="E11" s="46" t="n">
+      <c r="E12" s="53" t="n">
         <v>3.5</v>
       </c>
-      <c r="F11" s="27" t="n">
+      <c r="F12" s="27" t="n">
         <v>180</v>
       </c>
-      <c r="G11" s="28" t="n">
+      <c r="G12" s="28" t="n">
         <v>630</v>
       </c>
-      <c r="H11" s="25" t="inlineStr">
+      <c r="H12" s="25" t="inlineStr">
         <is>
           <t>Укладка сетки в слой стяжки</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="38" customHeight="1">
-      <c r="A12" s="30" t="n">
+    <row r="13" ht="38" customHeight="1">
+      <c r="A13" s="30" t="n">
         <v>8</v>
       </c>
-      <c r="B12" s="31" t="inlineStr">
+      <c r="B13" s="31" t="inlineStr">
         <is>
           <t>Устройство стяжки по маякам</t>
         </is>
       </c>
-      <c r="C12" s="31" t="inlineStr">
+      <c r="C13" s="31" t="inlineStr">
         <is>
           <t>Площадь пола ≈ 3,5 м²</t>
         </is>
       </c>
-      <c r="D12" s="30" t="inlineStr">
+      <c r="D13" s="30" t="inlineStr">
         <is>
           <t>м²</t>
         </is>
       </c>
-      <c r="E12" s="47" t="n">
+      <c r="E13" s="54" t="n">
         <v>3.5</v>
       </c>
-      <c r="F12" s="33" t="n">
+      <c r="F13" s="33" t="n">
         <v>350</v>
       </c>
-      <c r="G12" s="34" t="n">
+      <c r="G13" s="34" t="n">
         <v>1225</v>
       </c>
-      <c r="H12" s="31" t="inlineStr">
+      <c r="H13" s="31" t="inlineStr">
         <is>
           <t>Среднее 250–400 ₽/м², маяки в работе</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="38" customHeight="1">
-      <c r="A13" s="24" t="n">
+    <row r="14" ht="38" customHeight="1">
+      <c r="A14" s="24" t="n">
         <v>9</v>
       </c>
-      <c r="B13" s="25" t="inlineStr">
-        <is>
-          <t>Монтаж подоконника 1500×200 мм, пена, заглушка</t>
-        </is>
-      </c>
-      <c r="C13" s="25" t="inlineStr">
-        <is>
-          <t>Подоконник 1,5 м</t>
-        </is>
-      </c>
-      <c r="D13" s="24" t="inlineStr">
-        <is>
-          <t>п.м.</t>
-        </is>
-      </c>
-      <c r="E13" s="46" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="F13" s="27" t="n">
-        <v>600</v>
-      </c>
-      <c r="G13" s="28" t="n">
-        <v>900</v>
-      </c>
-      <c r="H13" s="25" t="inlineStr">
-        <is>
-          <t>Среднее по Краснодару около 600 ₽/п.м.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="38" customHeight="1">
-      <c r="A14" s="30" t="n">
+      <c r="B14" s="25" t="inlineStr">
+        <is>
+          <t>Подъём материалов, текущая уборка рабочей зоны</t>
+        </is>
+      </c>
+      <c r="C14" s="25" t="inlineStr">
+        <is>
+          <t>Комплект балкона 1</t>
+        </is>
+      </c>
+      <c r="D14" s="24" t="inlineStr">
+        <is>
+          <t>компл.</t>
+        </is>
+      </c>
+      <c r="E14" s="53" t="n">
+        <v>1</v>
+      </c>
+      <c r="F14" s="27" t="n">
+        <v>2500</v>
+      </c>
+      <c r="G14" s="28" t="n">
+        <v>2500</v>
+      </c>
+      <c r="H14" s="25" t="inlineStr">
+        <is>
+          <t>Не включает вывоз мусора — см. исключения</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="24" customHeight="1">
+      <c r="A15" s="49" t="inlineStr">
+        <is>
+          <t>ИТОГО ПО ЭТОМУ БАЛКОНУ</t>
+        </is>
+      </c>
+      <c r="B15" s="50" t="n"/>
+      <c r="C15" s="50" t="n"/>
+      <c r="D15" s="50" t="n"/>
+      <c r="E15" s="50" t="n"/>
+      <c r="F15" s="50" t="n"/>
+      <c r="G15" s="51">
+        <f>SUM(G6:G14)</f>
+        <v/>
+      </c>
+      <c r="H15" s="5" t="n"/>
+    </row>
+    <row r="17" ht="22" customHeight="1">
+      <c r="A17" s="52" t="inlineStr">
+        <is>
+          <t>БАЛКОН 2</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="n"/>
+      <c r="C17" s="7" t="n"/>
+      <c r="D17" s="7" t="n"/>
+      <c r="E17" s="7" t="n"/>
+      <c r="F17" s="7" t="n"/>
+      <c r="G17" s="7" t="n"/>
+      <c r="H17" s="7" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="23" t="inlineStr">
+        <is>
+          <t>№</t>
+        </is>
+      </c>
+      <c r="B18" s="23" t="inlineStr">
+        <is>
+          <t>Вид работ</t>
+        </is>
+      </c>
+      <c r="C18" s="23" t="inlineStr">
+        <is>
+          <t>Обоснование объёма</t>
+        </is>
+      </c>
+      <c r="D18" s="23" t="inlineStr">
+        <is>
+          <t>Ед.</t>
+        </is>
+      </c>
+      <c r="E18" s="23" t="inlineStr">
+        <is>
+          <t>Кол-во</t>
+        </is>
+      </c>
+      <c r="F18" s="23" t="inlineStr">
+        <is>
+          <t>Ставка, ₽</t>
+        </is>
+      </c>
+      <c r="G18" s="23" t="inlineStr">
+        <is>
+          <t>Сумма, ₽</t>
+        </is>
+      </c>
+      <c r="H18" s="23" t="inlineStr">
+        <is>
+          <t>Примечание</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="38" customHeight="1">
+      <c r="A19" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="B19" s="25" t="inlineStr">
+        <is>
+          <t>Каркас из ППН 27/28 и ПП 60/27, обшивка ГКЛ 12,5 мм</t>
+        </is>
+      </c>
+      <c r="C19" s="25" t="inlineStr">
+        <is>
+          <t>3 листа ГКЛ × 3 м² = 9,0 м²</t>
+        </is>
+      </c>
+      <c r="D19" s="24" t="inlineStr">
+        <is>
+          <t>м²</t>
+        </is>
+      </c>
+      <c r="E19" s="53" t="n">
+        <v>9</v>
+      </c>
+      <c r="F19" s="27" t="n">
+        <v>650</v>
+      </c>
+      <c r="G19" s="28" t="n">
+        <v>5850</v>
+      </c>
+      <c r="H19" s="25" t="inlineStr">
+        <is>
+          <t>Те же ставки, что на балконе 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="38" customHeight="1">
+      <c r="A20" s="30" t="n">
+        <v>2</v>
+      </c>
+      <c r="B20" s="31" t="inlineStr">
+        <is>
+          <t>Утепление каркаса минеральной ватой 50 мм</t>
+        </is>
+      </c>
+      <c r="C20" s="31" t="inlineStr">
+        <is>
+          <t>Площадь обшивки ГКЛ 9,0 м², 1 упаковка Тисма</t>
+        </is>
+      </c>
+      <c r="D20" s="30" t="inlineStr">
+        <is>
+          <t>м²</t>
+        </is>
+      </c>
+      <c r="E20" s="54" t="n">
+        <v>9</v>
+      </c>
+      <c r="F20" s="33" t="n">
+        <v>450</v>
+      </c>
+      <c r="G20" s="34" t="n">
+        <v>4050</v>
+      </c>
+      <c r="H20" s="31" t="inlineStr">
+        <is>
+          <t>Работа без материала</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="38" customHeight="1">
+      <c r="A21" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="B21" s="25" t="inlineStr">
+        <is>
+          <t>Заделка швов бумажной лентой, шпаклёвка под покраску</t>
+        </is>
+      </c>
+      <c r="C21" s="25" t="inlineStr">
+        <is>
+          <t>Площадь ГКЛ 9,0 м²</t>
+        </is>
+      </c>
+      <c r="D21" s="24" t="inlineStr">
+        <is>
+          <t>м²</t>
+        </is>
+      </c>
+      <c r="E21" s="53" t="n">
+        <v>9</v>
+      </c>
+      <c r="F21" s="27" t="n">
+        <v>380</v>
+      </c>
+      <c r="G21" s="28" t="n">
+        <v>3420</v>
+      </c>
+      <c r="H21" s="25" t="inlineStr">
+        <is>
+          <t>Материал общий из корзины, работа на этом балконе</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="38" customHeight="1">
+      <c r="A22" s="30" t="n">
+        <v>4</v>
+      </c>
+      <c r="B22" s="31" t="inlineStr">
+        <is>
+          <t>Грунтовка интерьерная, 2 раза</t>
+        </is>
+      </c>
+      <c r="C22" s="31" t="inlineStr">
+        <is>
+          <t>Площадь ГКЛ 9,0 м²</t>
+        </is>
+      </c>
+      <c r="D22" s="30" t="inlineStr">
+        <is>
+          <t>м²</t>
+        </is>
+      </c>
+      <c r="E22" s="54" t="n">
+        <v>9</v>
+      </c>
+      <c r="F22" s="33" t="n">
+        <v>120</v>
+      </c>
+      <c r="G22" s="34" t="n">
+        <v>1080</v>
+      </c>
+      <c r="H22" s="31" t="inlineStr">
+        <is>
+          <t>По 60 ₽/м² за проход</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="38" customHeight="1">
+      <c r="A23" s="24" t="n">
+        <v>5</v>
+      </c>
+      <c r="B23" s="25" t="inlineStr">
+        <is>
+          <t>Покраска стен/потолка, 2 слоя</t>
+        </is>
+      </c>
+      <c r="C23" s="25" t="inlineStr">
+        <is>
+          <t>Площадь ГКЛ 9,0 м²</t>
+        </is>
+      </c>
+      <c r="D23" s="24" t="inlineStr">
+        <is>
+          <t>м²</t>
+        </is>
+      </c>
+      <c r="E23" s="53" t="n">
+        <v>9</v>
+      </c>
+      <c r="F23" s="27" t="n">
+        <v>260</v>
+      </c>
+      <c r="G23" s="28" t="n">
+        <v>2340</v>
+      </c>
+      <c r="H23" s="25" t="inlineStr">
+        <is>
+          <t>Материал общий из корзины, работа на этом балконе</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="38" customHeight="1">
+      <c r="A24" s="30" t="n">
+        <v>6</v>
+      </c>
+      <c r="B24" s="31" t="inlineStr">
+        <is>
+          <t>Утепление пола Пеноплэксом 50 мм, крепление пресс-шайбой</t>
+        </is>
+      </c>
+      <c r="C24" s="31" t="inlineStr">
+        <is>
+          <t>5 листов × 0,69 м² ≈ 3,5 м²</t>
+        </is>
+      </c>
+      <c r="D24" s="30" t="inlineStr">
+        <is>
+          <t>м²</t>
+        </is>
+      </c>
+      <c r="E24" s="54" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="F24" s="33" t="n">
+        <v>400</v>
+      </c>
+      <c r="G24" s="34" t="n">
+        <v>1400</v>
+      </c>
+      <c r="H24" s="31" t="inlineStr">
+        <is>
+          <t>Во втором списке грибов нет, крепёж пресс-шайбой</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="38" customHeight="1">
+      <c r="A25" s="24" t="n">
+        <v>7</v>
+      </c>
+      <c r="B25" s="25" t="inlineStr">
+        <is>
+          <t>Армирование стяжки стеклопластиковой сеткой 50×50</t>
+        </is>
+      </c>
+      <c r="C25" s="25" t="inlineStr">
+        <is>
+          <t>Площадь пола ≈ 3,5 м²</t>
+        </is>
+      </c>
+      <c r="D25" s="24" t="inlineStr">
+        <is>
+          <t>м²</t>
+        </is>
+      </c>
+      <c r="E25" s="53" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="F25" s="27" t="n">
+        <v>180</v>
+      </c>
+      <c r="G25" s="28" t="n">
+        <v>630</v>
+      </c>
+      <c r="H25" s="25" t="inlineStr">
+        <is>
+          <t>Укладка сетки в слой стяжки</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="38" customHeight="1">
+      <c r="A26" s="30" t="n">
+        <v>8</v>
+      </c>
+      <c r="B26" s="31" t="inlineStr">
+        <is>
+          <t>Устройство стяжки по маякам</t>
+        </is>
+      </c>
+      <c r="C26" s="31" t="inlineStr">
+        <is>
+          <t>Площадь пола ≈ 3,5 м²</t>
+        </is>
+      </c>
+      <c r="D26" s="30" t="inlineStr">
+        <is>
+          <t>м²</t>
+        </is>
+      </c>
+      <c r="E26" s="54" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="F26" s="33" t="n">
+        <v>350</v>
+      </c>
+      <c r="G26" s="34" t="n">
+        <v>1225</v>
+      </c>
+      <c r="H26" s="31" t="inlineStr">
+        <is>
+          <t>Маяки в работе</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="38" customHeight="1">
+      <c r="A27" s="24" t="n">
+        <v>9</v>
+      </c>
+      <c r="B27" s="25" t="inlineStr">
+        <is>
+          <t>Подъём материалов, текущая уборка рабочей зоны</t>
+        </is>
+      </c>
+      <c r="C27" s="25" t="inlineStr">
+        <is>
+          <t>Комплект балкона 2</t>
+        </is>
+      </c>
+      <c r="D27" s="24" t="inlineStr">
+        <is>
+          <t>компл.</t>
+        </is>
+      </c>
+      <c r="E27" s="53" t="n">
+        <v>1</v>
+      </c>
+      <c r="F27" s="27" t="n">
+        <v>2500</v>
+      </c>
+      <c r="G27" s="28" t="n">
+        <v>2500</v>
+      </c>
+      <c r="H27" s="25" t="inlineStr">
+        <is>
+          <t>Если оба балкона в одну поездку, два подъёма могут сойтись чуть дешевле</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="24" customHeight="1">
+      <c r="A28" s="49" t="inlineStr">
+        <is>
+          <t>ИТОГО ПО ЭТОМУ БАЛКОНУ</t>
+        </is>
+      </c>
+      <c r="B28" s="50" t="n"/>
+      <c r="C28" s="50" t="n"/>
+      <c r="D28" s="50" t="n"/>
+      <c r="E28" s="50" t="n"/>
+      <c r="F28" s="50" t="n"/>
+      <c r="G28" s="51">
+        <f>SUM(G19:G27)</f>
+        <v/>
+      </c>
+      <c r="H28" s="5" t="n"/>
+    </row>
+    <row r="30" ht="26" customHeight="1">
+      <c r="A30" s="55" t="inlineStr">
+        <is>
+          <t>ИТОГО РАБОТЫ, ОБА БАЛКОНА</t>
+        </is>
+      </c>
+      <c r="B30" s="56" t="n"/>
+      <c r="C30" s="56" t="n"/>
+      <c r="D30" s="56" t="n"/>
+      <c r="E30" s="56" t="n"/>
+      <c r="F30" s="56" t="n"/>
+      <c r="G30" s="51">
+        <f>G15+G28</f>
+        <v/>
+      </c>
+      <c r="H30" s="9" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="14" t="inlineStr">
+        <is>
+          <t>НЕ ВХОДИТ В ЭТУ СМЕТУ РАБОТ</t>
+        </is>
+      </c>
+      <c r="B32" s="15" t="n"/>
+      <c r="C32" s="15" t="n"/>
+      <c r="D32" s="15" t="n"/>
+      <c r="E32" s="15" t="n"/>
+      <c r="F32" s="15" t="n"/>
+      <c r="G32" s="15" t="n"/>
+      <c r="H32" s="15" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="57" t="inlineStr">
+        <is>
+          <t>№</t>
+        </is>
+      </c>
+      <c r="B33" s="57" t="inlineStr">
+        <is>
+          <t>Что не входит</t>
+        </is>
+      </c>
+      <c r="C33" s="57" t="inlineStr">
+        <is>
+          <t>Почему не входит</t>
+        </is>
+      </c>
+      <c r="D33" s="57" t="inlineStr">
+        <is>
+          <t>Как обычно считают</t>
+        </is>
+      </c>
+      <c r="E33" s="58" t="n"/>
+      <c r="F33" s="58" t="n"/>
+      <c r="G33" s="58" t="n"/>
+      <c r="H33" s="58" t="n"/>
+    </row>
+    <row r="34" ht="32" customHeight="1">
+      <c r="A34" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="B34" s="60" t="inlineStr">
+        <is>
+          <t>Демонтаж старой отделки, старой стяжки, подоконника и обшивки</t>
+        </is>
+      </c>
+      <c r="C34" s="60" t="inlineStr">
+        <is>
+          <t>В списках материалов нет позиций на демонтаж</t>
+        </is>
+      </c>
+      <c r="D34" s="60" t="inlineStr">
+        <is>
+          <t>Отдельно, обычно 150–350 ₽/м² в зависимости от слоя</t>
+        </is>
+      </c>
+      <c r="E34" s="61" t="n"/>
+      <c r="F34" s="61" t="n"/>
+      <c r="G34" s="61" t="n"/>
+      <c r="H34" s="61" t="n"/>
+    </row>
+    <row r="35" ht="32" customHeight="1">
+      <c r="A35" s="59" t="n">
+        <v>2</v>
+      </c>
+      <c r="B35" s="60" t="inlineStr">
+        <is>
+          <t>Остекление балкона, замена окна, монтаж откосов, отлива и подоконника</t>
+        </is>
+      </c>
+      <c r="C35" s="60" t="inlineStr">
+        <is>
+          <t>Подоконники не делаются, остекления в смете нет</t>
+        </is>
+      </c>
+      <c r="D35" s="60" t="inlineStr">
+        <is>
+          <t>Отдельный договор на остекление</t>
+        </is>
+      </c>
+      <c r="E35" s="61" t="n"/>
+      <c r="F35" s="61" t="n"/>
+      <c r="G35" s="61" t="n"/>
+      <c r="H35" s="61" t="n"/>
+    </row>
+    <row r="36" ht="32" customHeight="1">
+      <c r="A36" s="59" t="n">
+        <v>3</v>
+      </c>
+      <c r="B36" s="60" t="inlineStr">
+        <is>
+          <t>Электромонтаж: кабель, розетки, светильники, тёплый пол</t>
+        </is>
+      </c>
+      <c r="C36" s="60" t="inlineStr">
+        <is>
+          <t>В списке нет кабеля, коробок, тёплого пола</t>
+        </is>
+      </c>
+      <c r="D36" s="60" t="inlineStr">
+        <is>
+          <t>Отдельная смета электрика</t>
+        </is>
+      </c>
+      <c r="E36" s="61" t="n"/>
+      <c r="F36" s="61" t="n"/>
+      <c r="G36" s="61" t="n"/>
+      <c r="H36" s="61" t="n"/>
+    </row>
+    <row r="37" ht="32" customHeight="1">
+      <c r="A37" s="59" t="n">
+        <v>4</v>
+      </c>
+      <c r="B37" s="60" t="inlineStr">
+        <is>
+          <t>Чистовой пол: плитка, ламинат, линолеум, плинтус, порожек</t>
+        </is>
+      </c>
+      <c r="C37" s="60" t="inlineStr">
+        <is>
+          <t>В материалах только черновая стяжка</t>
+        </is>
+      </c>
+      <c r="D37" s="60" t="inlineStr">
+        <is>
+          <t>Плитка от 900 ₽/м², ламинат от 350 ₽/м² работа</t>
+        </is>
+      </c>
+      <c r="E37" s="61" t="n"/>
+      <c r="F37" s="61" t="n"/>
+      <c r="G37" s="61" t="n"/>
+      <c r="H37" s="61" t="n"/>
+    </row>
+    <row r="38" ht="32" customHeight="1">
+      <c r="A38" s="59" t="n">
+        <v>5</v>
+      </c>
+      <c r="B38" s="60" t="inlineStr">
+        <is>
+          <t>Гидроизоляция пола и парапета, пароизоляция, фольгированный слой</t>
+        </is>
+      </c>
+      <c r="C38" s="60" t="inlineStr">
+        <is>
+          <t>В списке нет рулонной гидро- и пароизоляции</t>
+        </is>
+      </c>
+      <c r="D38" s="60" t="inlineStr">
+        <is>
+          <t>Отдельно 150–250 ₽/м²</t>
+        </is>
+      </c>
+      <c r="E38" s="61" t="n"/>
+      <c r="F38" s="61" t="n"/>
+      <c r="G38" s="61" t="n"/>
+      <c r="H38" s="61" t="n"/>
+    </row>
+    <row r="39" ht="32" customHeight="1">
+      <c r="A39" s="59" t="n">
+        <v>6</v>
+      </c>
+      <c r="B39" s="60" t="inlineStr">
+        <is>
+          <t>Доставка материалов из Лемана ПРО и подъём грузчиками магазина</t>
+        </is>
+      </c>
+      <c r="C39" s="60" t="inlineStr">
+        <is>
+          <t>В работах только подъём на объект силами бригады</t>
+        </is>
+      </c>
+      <c r="D39" s="60" t="inlineStr">
+        <is>
+          <t>По тарифу магазина / такси</t>
+        </is>
+      </c>
+      <c r="E39" s="61" t="n"/>
+      <c r="F39" s="61" t="n"/>
+      <c r="G39" s="61" t="n"/>
+      <c r="H39" s="61" t="n"/>
+    </row>
+    <row r="40" ht="32" customHeight="1">
+      <c r="A40" s="59" t="n">
+        <v>7</v>
+      </c>
+      <c r="B40" s="60" t="inlineStr">
+        <is>
+          <t>Вывоз строительного мусора, контейнер, погрузка</t>
+        </is>
+      </c>
+      <c r="C40" s="60" t="inlineStr">
+        <is>
+          <t>В п. 9 каждого балкона только текущая уборка зоны</t>
+        </is>
+      </c>
+      <c r="D40" s="60" t="inlineStr">
+        <is>
+          <t>Контейнер / Газель отдельно</t>
+        </is>
+      </c>
+      <c r="E40" s="61" t="n"/>
+      <c r="F40" s="61" t="n"/>
+      <c r="G40" s="61" t="n"/>
+      <c r="H40" s="61" t="n"/>
+    </row>
+    <row r="41" ht="32" customHeight="1">
+      <c r="A41" s="59" t="n">
+        <v>8</v>
+      </c>
+      <c r="B41" s="60" t="inlineStr">
+        <is>
+          <t>Наружная отделка ограждения, фасад, козырёк, москитные сетки</t>
+        </is>
+      </c>
+      <c r="C41" s="60" t="inlineStr">
+        <is>
+          <t>Материалы только на внутренний контур балкона</t>
+        </is>
+      </c>
+      <c r="D41" s="60" t="inlineStr">
+        <is>
+          <t>Отдельный вид работ</t>
+        </is>
+      </c>
+      <c r="E41" s="61" t="n"/>
+      <c r="F41" s="61" t="n"/>
+      <c r="G41" s="61" t="n"/>
+      <c r="H41" s="61" t="n"/>
+    </row>
+    <row r="42" ht="32" customHeight="1">
+      <c r="A42" s="59" t="n">
+        <v>9</v>
+      </c>
+      <c r="B42" s="60" t="inlineStr">
+        <is>
+          <t>Согласование перепланировки, технадзор, скрытые работы</t>
+        </is>
+      </c>
+      <c r="C42" s="60" t="inlineStr">
+        <is>
+          <t>Не заказывались и не оценивались</t>
+        </is>
+      </c>
+      <c r="D42" s="60" t="inlineStr">
+        <is>
+          <t>По факту после вскрытия</t>
+        </is>
+      </c>
+      <c r="E42" s="61" t="n"/>
+      <c r="F42" s="61" t="n"/>
+      <c r="G42" s="61" t="n"/>
+      <c r="H42" s="61" t="n"/>
+    </row>
+    <row r="43" ht="32" customHeight="1">
+      <c r="A43" s="59" t="n">
         <v>10</v>
       </c>
-      <c r="B14" s="31" t="inlineStr">
-        <is>
-          <t>Подъём материалов на объект, текущая уборка рабочей зоны</t>
-        </is>
-      </c>
-      <c r="C14" s="31" t="inlineStr">
-        <is>
-          <t>Комплект по смете материалов</t>
-        </is>
-      </c>
-      <c r="D14" s="30" t="inlineStr">
-        <is>
-          <t>компл.</t>
-        </is>
-      </c>
-      <c r="E14" s="47" t="n">
-        <v>1</v>
-      </c>
-      <c r="F14" s="33" t="n">
-        <v>2500</v>
-      </c>
-      <c r="G14" s="34" t="n">
-        <v>2500</v>
-      </c>
-      <c r="H14" s="31" t="inlineStr">
-        <is>
-          <t>Не включает вывоз мусора с объекта — см. исключения</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="24" customHeight="1">
-      <c r="A15" s="43" t="inlineStr">
-        <is>
-          <t>ИТОГО РАБОТЫ</t>
-        </is>
-      </c>
-      <c r="B15" s="44" t="n"/>
-      <c r="C15" s="44" t="n"/>
-      <c r="D15" s="44" t="n"/>
-      <c r="E15" s="44" t="n"/>
-      <c r="F15" s="44" t="n"/>
-      <c r="G15" s="45">
-        <f>SUM(G5:G14)</f>
-        <v/>
-      </c>
-      <c r="H15" s="5" t="n"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="14" t="inlineStr">
-        <is>
-          <t>НЕ ВХОДИТ В ЭТУ СМЕТУ РАБОТ</t>
-        </is>
-      </c>
-      <c r="B17" s="15" t="n"/>
-      <c r="C17" s="15" t="n"/>
-      <c r="D17" s="15" t="n"/>
-      <c r="E17" s="15" t="n"/>
-      <c r="F17" s="15" t="n"/>
-      <c r="G17" s="15" t="n"/>
-      <c r="H17" s="15" t="n"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="48" t="inlineStr">
-        <is>
-          <t>№</t>
-        </is>
-      </c>
-      <c r="B18" s="48" t="inlineStr">
-        <is>
-          <t>Что не входит</t>
-        </is>
-      </c>
-      <c r="C18" s="48" t="inlineStr">
-        <is>
-          <t>Почему не входит</t>
-        </is>
-      </c>
-      <c r="D18" s="48" t="inlineStr">
-        <is>
-          <t>Как обычно считают</t>
-        </is>
-      </c>
-      <c r="E18" s="49" t="n"/>
-      <c r="F18" s="49" t="n"/>
-      <c r="G18" s="49" t="n"/>
-      <c r="H18" s="49" t="n"/>
-    </row>
-    <row r="19" ht="32" customHeight="1">
-      <c r="A19" s="50" t="n">
-        <v>1</v>
-      </c>
-      <c r="B19" s="51" t="inlineStr">
-        <is>
-          <t>Демонтаж старой отделки, старой стяжки, старого подоконника и обшивки</t>
-        </is>
-      </c>
-      <c r="C19" s="51" t="inlineStr">
-        <is>
-          <t>В списке материалов нет позиций на демонтаж</t>
-        </is>
-      </c>
-      <c r="D19" s="51" t="inlineStr">
-        <is>
-          <t>Отдельно, обычно 150–350 ₽/м² в зависимости от слоя</t>
-        </is>
-      </c>
-      <c r="E19" s="52" t="n"/>
-      <c r="F19" s="52" t="n"/>
-      <c r="G19" s="52" t="n"/>
-      <c r="H19" s="52" t="n"/>
-    </row>
-    <row r="20" ht="32" customHeight="1">
-      <c r="A20" s="50" t="n">
-        <v>2</v>
-      </c>
-      <c r="B20" s="51" t="inlineStr">
-        <is>
-          <t>Остекление балкона, замена окна, монтаж откосов и отлива</t>
-        </is>
-      </c>
-      <c r="C20" s="51" t="inlineStr">
-        <is>
-          <t>В материалах только подоконник, окна нет</t>
-        </is>
-      </c>
-      <c r="D20" s="51" t="inlineStr">
-        <is>
-          <t>Отдельный договор на остекление</t>
-        </is>
-      </c>
-      <c r="E20" s="52" t="n"/>
-      <c r="F20" s="52" t="n"/>
-      <c r="G20" s="52" t="n"/>
-      <c r="H20" s="52" t="n"/>
-    </row>
-    <row r="21" ht="32" customHeight="1">
-      <c r="A21" s="50" t="n">
-        <v>3</v>
-      </c>
-      <c r="B21" s="51" t="inlineStr">
-        <is>
-          <t>Электромонтаж: кабель, розетки, светильники, тёплый пол</t>
-        </is>
-      </c>
-      <c r="C21" s="51" t="inlineStr">
-        <is>
-          <t>В списке нет кабеля, коробок, тёплого пола</t>
-        </is>
-      </c>
-      <c r="D21" s="51" t="inlineStr">
-        <is>
-          <t>Отдельная смета электрика</t>
-        </is>
-      </c>
-      <c r="E21" s="52" t="n"/>
-      <c r="F21" s="52" t="n"/>
-      <c r="G21" s="52" t="n"/>
-      <c r="H21" s="52" t="n"/>
-    </row>
-    <row r="22" ht="32" customHeight="1">
-      <c r="A22" s="50" t="n">
-        <v>4</v>
-      </c>
-      <c r="B22" s="51" t="inlineStr">
-        <is>
-          <t>Чистовой пол: плитка, ламинат, линолеум, плинтус, порожек</t>
-        </is>
-      </c>
-      <c r="C22" s="51" t="inlineStr">
-        <is>
-          <t>В материалах только черновая стяжка</t>
-        </is>
-      </c>
-      <c r="D22" s="51" t="inlineStr">
-        <is>
-          <t>Плитка от 900 ₽/м², ламинат от 350 ₽/м² работа</t>
-        </is>
-      </c>
-      <c r="E22" s="52" t="n"/>
-      <c r="F22" s="52" t="n"/>
-      <c r="G22" s="52" t="n"/>
-      <c r="H22" s="52" t="n"/>
-    </row>
-    <row r="23" ht="32" customHeight="1">
-      <c r="A23" s="50" t="n">
-        <v>5</v>
-      </c>
-      <c r="B23" s="51" t="inlineStr">
-        <is>
-          <t>Гидроизоляция пола и парапета, пароизоляция, фольгированный слой</t>
-        </is>
-      </c>
-      <c r="C23" s="51" t="inlineStr">
-        <is>
-          <t>В списке нет рулонной гидро- и пароизоляции</t>
-        </is>
-      </c>
-      <c r="D23" s="51" t="inlineStr">
-        <is>
-          <t>Отдельно 150–250 ₽/м²</t>
-        </is>
-      </c>
-      <c r="E23" s="52" t="n"/>
-      <c r="F23" s="52" t="n"/>
-      <c r="G23" s="52" t="n"/>
-      <c r="H23" s="52" t="n"/>
-    </row>
-    <row r="24" ht="32" customHeight="1">
-      <c r="A24" s="50" t="n">
-        <v>6</v>
-      </c>
-      <c r="B24" s="51" t="inlineStr">
-        <is>
-          <t>Доставка материалов из Лемана ПРО и подъём грузчиками магазина</t>
-        </is>
-      </c>
-      <c r="C24" s="51" t="inlineStr">
-        <is>
-          <t>В работах только подъём на объект силами бригады</t>
-        </is>
-      </c>
-      <c r="D24" s="51" t="inlineStr">
-        <is>
-          <t>По тарифу магазина / такси</t>
-        </is>
-      </c>
-      <c r="E24" s="52" t="n"/>
-      <c r="F24" s="52" t="n"/>
-      <c r="G24" s="52" t="n"/>
-      <c r="H24" s="52" t="n"/>
-    </row>
-    <row r="25" ht="32" customHeight="1">
-      <c r="A25" s="50" t="n">
-        <v>7</v>
-      </c>
-      <c r="B25" s="51" t="inlineStr">
-        <is>
-          <t>Вывоз строительного мусора, контейнер, погрузка</t>
-        </is>
-      </c>
-      <c r="C25" s="51" t="inlineStr">
-        <is>
-          <t>В п. 10 только текущая уборка рабочей зоны</t>
-        </is>
-      </c>
-      <c r="D25" s="51" t="inlineStr">
-        <is>
-          <t>Контейнер / Газель отдельно</t>
-        </is>
-      </c>
-      <c r="E25" s="52" t="n"/>
-      <c r="F25" s="52" t="n"/>
-      <c r="G25" s="52" t="n"/>
-      <c r="H25" s="52" t="n"/>
-    </row>
-    <row r="26" ht="32" customHeight="1">
-      <c r="A26" s="50" t="n">
-        <v>8</v>
-      </c>
-      <c r="B26" s="51" t="inlineStr">
-        <is>
-          <t>Наружная отделка ограждения, фасад, козырёк, москитные сетки</t>
-        </is>
-      </c>
-      <c r="C26" s="51" t="inlineStr">
-        <is>
-          <t>Материалы только на внутренний контур балкона</t>
-        </is>
-      </c>
-      <c r="D26" s="51" t="inlineStr">
-        <is>
-          <t>Отдельный вид работ</t>
-        </is>
-      </c>
-      <c r="E26" s="52" t="n"/>
-      <c r="F26" s="52" t="n"/>
-      <c r="G26" s="52" t="n"/>
-      <c r="H26" s="52" t="n"/>
-    </row>
-    <row r="27" ht="32" customHeight="1">
-      <c r="A27" s="50" t="n">
-        <v>9</v>
-      </c>
-      <c r="B27" s="51" t="inlineStr">
-        <is>
-          <t>Согласование перепланировки, технадзор, скрытые работы</t>
-        </is>
-      </c>
-      <c r="C27" s="51" t="inlineStr">
-        <is>
-          <t>Не заказывались и не оценивались</t>
-        </is>
-      </c>
-      <c r="D27" s="51" t="inlineStr">
-        <is>
-          <t>По факту после вскрытия</t>
-        </is>
-      </c>
-      <c r="E27" s="52" t="n"/>
-      <c r="F27" s="52" t="n"/>
-      <c r="G27" s="52" t="n"/>
-      <c r="H27" s="52" t="n"/>
-    </row>
-    <row r="28" ht="32" customHeight="1">
-      <c r="A28" s="50" t="n">
-        <v>10</v>
-      </c>
-      <c r="B28" s="51" t="inlineStr">
+      <c r="B43" s="60" t="inlineStr">
         <is>
           <t>Повторная покраска сверх 2 слоёв, колеровка, декоративные покрытия</t>
         </is>
       </c>
-      <c r="C28" s="51" t="inlineStr">
-        <is>
-          <t>В смете 2 слоя обычной интерьерной краски</t>
-        </is>
-      </c>
-      <c r="D28" s="51" t="inlineStr">
+      <c r="C43" s="60" t="inlineStr">
+        <is>
+          <t>В смете 2 слоя обычной интерьерной краски на каждый балкон</t>
+        </is>
+      </c>
+      <c r="D43" s="60" t="inlineStr">
         <is>
           <t>Доп. слой ~120–150 ₽/м²</t>
         </is>
       </c>
-      <c r="E28" s="52" t="n"/>
-      <c r="F28" s="52" t="n"/>
-      <c r="G28" s="52" t="n"/>
-      <c r="H28" s="52" t="n"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="53" t="inlineStr">
-        <is>
-          <t>Итог работ 23 395 ₽ действует только на перечень строк 1–10. Всё, что в красном блоке, в эту сумму не входит и оценивается отдельно после замера.</t>
-        </is>
-      </c>
-      <c r="B30" s="54" t="n"/>
-      <c r="C30" s="54" t="n"/>
-      <c r="D30" s="54" t="n"/>
-      <c r="E30" s="54" t="n"/>
-      <c r="F30" s="54" t="n"/>
-      <c r="G30" s="54" t="n"/>
-      <c r="H30" s="54" t="n"/>
-    </row>
-    <row r="31">
-      <c r="A31" s="54" t="n"/>
-      <c r="B31" s="54" t="n"/>
-      <c r="C31" s="54" t="n"/>
-      <c r="D31" s="54" t="n"/>
-      <c r="E31" s="54" t="n"/>
-      <c r="F31" s="54" t="n"/>
-      <c r="G31" s="54" t="n"/>
-      <c r="H31" s="54" t="n"/>
+      <c r="E43" s="61" t="n"/>
+      <c r="F43" s="61" t="n"/>
+      <c r="G43" s="61" t="n"/>
+      <c r="H43" s="61" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="62" t="inlineStr">
+        <is>
+          <t>Итог работ 44 990 ₽ = 22 495 ₽ × 2 балкона, только строки 1–9 на каждом. Всё, что в красном блоке, в эту сумму не входит и оценивается отдельно после замера. Если оба балкона в одну поездку, два подъёма по 2 500 ₽ могут сойтись чуть дешевле.</t>
+        </is>
+      </c>
+      <c r="B45" s="63" t="n"/>
+      <c r="C45" s="63" t="n"/>
+      <c r="D45" s="63" t="n"/>
+      <c r="E45" s="63" t="n"/>
+      <c r="F45" s="63" t="n"/>
+      <c r="G45" s="63" t="n"/>
+      <c r="H45" s="63" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="63" t="n"/>
+      <c r="B46" s="63" t="n"/>
+      <c r="C46" s="63" t="n"/>
+      <c r="D46" s="63" t="n"/>
+      <c r="E46" s="63" t="n"/>
+      <c r="F46" s="63" t="n"/>
+      <c r="G46" s="63" t="n"/>
+      <c r="H46" s="63" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A4:H14"/>
-  <mergeCells count="16">
-    <mergeCell ref="D21:H21"/>
-    <mergeCell ref="D25:H25"/>
-    <mergeCell ref="D20:H20"/>
-    <mergeCell ref="D24:H24"/>
+  <mergeCells count="20">
+    <mergeCell ref="D35:H35"/>
+    <mergeCell ref="D34:H34"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="D40:H40"/>
+    <mergeCell ref="D36:H36"/>
+    <mergeCell ref="D41:H41"/>
+    <mergeCell ref="A28:F28"/>
+    <mergeCell ref="D43:H43"/>
     <mergeCell ref="A2:H2"/>
-    <mergeCell ref="D19:H19"/>
-    <mergeCell ref="D28:H28"/>
-    <mergeCell ref="D27:H27"/>
-    <mergeCell ref="D23:H23"/>
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A30:H31"/>
-    <mergeCell ref="D22:H22"/>
-    <mergeCell ref="D18:H18"/>
+    <mergeCell ref="D37:H37"/>
+    <mergeCell ref="A32:H32"/>
+    <mergeCell ref="A30:F30"/>
     <mergeCell ref="A15:F15"/>
-    <mergeCell ref="D26:H26"/>
     <mergeCell ref="A17:H17"/>
+    <mergeCell ref="A4:H4"/>
+    <mergeCell ref="D39:H39"/>
+    <mergeCell ref="D42:H42"/>
+    <mergeCell ref="A45:H46"/>
+    <mergeCell ref="D33:H33"/>
+    <mergeCell ref="D38:H38"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="1" fitToWidth="1"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;LПервый балкон, Краснодар&amp;C13.10.2026&amp;R&amp;P из &amp;N</oddFooter>
+    <oddFooter>&amp;LДва балкона, Краснодар&amp;C13.10.2026&amp;R&amp;P из &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -3029,7 +3437,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="55" t="inlineStr">
+      <c r="A1" s="64" t="inlineStr">
         <is>
           <t>НЕ ВХОДИТ В СМЕТУ РАБОТ</t>
         </is>
@@ -3041,431 +3449,431 @@
       <c r="F1" s="15" t="n"/>
     </row>
     <row r="2" ht="22" customHeight="1">
-      <c r="A2" s="56" t="inlineStr">
-        <is>
-          <t>Этот лист — полный перечень того, что НЕ входит в 23 395 ₽ за работу. Если нужно — оценивается отдельной сметой после замера.</t>
+      <c r="A2" s="65" t="inlineStr">
+        <is>
+          <t>Этот лист — полный перечень того, что НЕ входит в 44 990 ₽ за работу на оба балкона. Если нужно — оценивается отдельной сметой после замера.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="48" t="inlineStr">
+      <c r="A4" s="57" t="inlineStr">
         <is>
           <t>№</t>
         </is>
       </c>
-      <c r="B4" s="48" t="inlineStr">
+      <c r="B4" s="57" t="inlineStr">
         <is>
           <t>Не входит</t>
         </is>
       </c>
-      <c r="C4" s="48" t="inlineStr">
+      <c r="C4" s="57" t="inlineStr">
         <is>
           <t>Почему не входит в эту смету</t>
         </is>
       </c>
-      <c r="D4" s="48" t="inlineStr">
+      <c r="D4" s="57" t="inlineStr">
         <is>
           <t>Типичная оценка в Краснодаре</t>
         </is>
       </c>
-      <c r="E4" s="48" t="inlineStr">
+      <c r="E4" s="57" t="inlineStr">
         <is>
           <t>Нужен ли материал сверх списка</t>
         </is>
       </c>
-      <c r="F4" s="48" t="inlineStr">
+      <c r="F4" s="57" t="inlineStr">
         <is>
           <t>Статус</t>
         </is>
       </c>
     </row>
     <row r="5" ht="40" customHeight="1">
-      <c r="A5" s="50" t="n">
+      <c r="A5" s="59" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="51" t="inlineStr">
+      <c r="B5" s="60" t="inlineStr">
         <is>
           <t>Демонтаж старой отделки, стяжки, подоконника, обшивки</t>
         </is>
       </c>
-      <c r="C5" s="51" t="inlineStr">
+      <c r="C5" s="60" t="inlineStr">
         <is>
           <t>В исходном списке нет материалов и объёмов на демонтаж</t>
         </is>
       </c>
-      <c r="D5" s="51" t="inlineStr">
+      <c r="D5" s="60" t="inlineStr">
         <is>
           <t>150–350 ₽/м² в зависимости от слоя</t>
         </is>
       </c>
-      <c r="E5" s="51" t="inlineStr">
+      <c r="E5" s="60" t="inlineStr">
         <is>
           <t>Нет, это только работа + вывоз</t>
         </is>
       </c>
-      <c r="F5" s="57" t="inlineStr">
+      <c r="F5" s="66" t="inlineStr">
         <is>
           <t>НЕ ВХОДИТ</t>
         </is>
       </c>
     </row>
     <row r="6" ht="40" customHeight="1">
-      <c r="A6" s="50" t="n">
+      <c r="A6" s="59" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="51" t="inlineStr">
-        <is>
-          <t>Остекление, замена окна, откосы, отлив</t>
-        </is>
-      </c>
-      <c r="C6" s="51" t="inlineStr">
-        <is>
-          <t>В материалах только подоконник 1,5 м</t>
-        </is>
-      </c>
-      <c r="D6" s="51" t="inlineStr">
+      <c r="B6" s="60" t="inlineStr">
+        <is>
+          <t>Остекление, замена окна, откосы, отлив, подоконник</t>
+        </is>
+      </c>
+      <c r="C6" s="60" t="inlineStr">
+        <is>
+          <t>Подоконники не делаются, остекления в смете нет</t>
+        </is>
+      </c>
+      <c r="D6" s="60" t="inlineStr">
         <is>
           <t>Отдельный договор, от нескольких тысяч за окно</t>
         </is>
       </c>
-      <c r="E6" s="51" t="inlineStr">
+      <c r="E6" s="60" t="inlineStr">
         <is>
           <t>Да, профиль/стеклопакеты отдельно</t>
         </is>
       </c>
-      <c r="F6" s="57" t="inlineStr">
+      <c r="F6" s="66" t="inlineStr">
         <is>
           <t>НЕ ВХОДИТ</t>
         </is>
       </c>
     </row>
     <row r="7" ht="40" customHeight="1">
-      <c r="A7" s="50" t="n">
+      <c r="A7" s="59" t="n">
         <v>3</v>
       </c>
-      <c r="B7" s="51" t="inlineStr">
+      <c r="B7" s="60" t="inlineStr">
         <is>
           <t>Электрика, свет, розетки, тёплый пол</t>
         </is>
       </c>
-      <c r="C7" s="51" t="inlineStr">
+      <c r="C7" s="60" t="inlineStr">
         <is>
           <t>Кабеля, коробок и нагревательного элемента в списке нет</t>
         </is>
       </c>
-      <c r="D7" s="51" t="inlineStr">
+      <c r="D7" s="60" t="inlineStr">
         <is>
           <t>Отдельная смета электрика</t>
         </is>
       </c>
-      <c r="E7" s="51" t="inlineStr">
+      <c r="E7" s="60" t="inlineStr">
         <is>
           <t>Да, кабель, автоматы, тёплый пол</t>
         </is>
       </c>
-      <c r="F7" s="57" t="inlineStr">
+      <c r="F7" s="66" t="inlineStr">
         <is>
           <t>НЕ ВХОДИТ</t>
         </is>
       </c>
     </row>
     <row r="8" ht="40" customHeight="1">
-      <c r="A8" s="50" t="n">
+      <c r="A8" s="59" t="n">
         <v>4</v>
       </c>
-      <c r="B8" s="51" t="inlineStr">
+      <c r="B8" s="60" t="inlineStr">
         <is>
           <t>Чистовой пол: плитка / ламинат / линолеум / плинтус</t>
         </is>
       </c>
-      <c r="C8" s="51" t="inlineStr">
+      <c r="C8" s="60" t="inlineStr">
         <is>
           <t>В материалах только черновая стяжка и маяки</t>
         </is>
       </c>
-      <c r="D8" s="51" t="inlineStr">
+      <c r="D8" s="60" t="inlineStr">
         <is>
           <t>Плитка от ~900 ₽/м², ламинат от ~350 ₽/м² работа</t>
         </is>
       </c>
-      <c r="E8" s="51" t="inlineStr">
+      <c r="E8" s="60" t="inlineStr">
         <is>
           <t>Да, покрытие и плинтус</t>
         </is>
       </c>
-      <c r="F8" s="57" t="inlineStr">
+      <c r="F8" s="66" t="inlineStr">
         <is>
           <t>НЕ ВХОДИТ</t>
         </is>
       </c>
     </row>
     <row r="9" ht="40" customHeight="1">
-      <c r="A9" s="50" t="n">
+      <c r="A9" s="59" t="n">
         <v>5</v>
       </c>
-      <c r="B9" s="51" t="inlineStr">
+      <c r="B9" s="60" t="inlineStr">
         <is>
           <t>Гидроизоляция пола и парапета, пароизоляция</t>
         </is>
       </c>
-      <c r="C9" s="51" t="inlineStr">
+      <c r="C9" s="60" t="inlineStr">
         <is>
           <t>Рулонной изоляции в списке нет</t>
         </is>
       </c>
-      <c r="D9" s="51" t="inlineStr">
+      <c r="D9" s="60" t="inlineStr">
         <is>
           <t>150–250 ₽/м² работа</t>
         </is>
       </c>
-      <c r="E9" s="51" t="inlineStr">
+      <c r="E9" s="60" t="inlineStr">
         <is>
           <t>Да, мембрана / мастика</t>
         </is>
       </c>
-      <c r="F9" s="57" t="inlineStr">
+      <c r="F9" s="66" t="inlineStr">
         <is>
           <t>НЕ ВХОДИТ</t>
         </is>
       </c>
     </row>
     <row r="10" ht="40" customHeight="1">
-      <c r="A10" s="50" t="n">
+      <c r="A10" s="59" t="n">
         <v>6</v>
       </c>
-      <c r="B10" s="51" t="inlineStr">
+      <c r="B10" s="60" t="inlineStr">
         <is>
           <t>Доставка из Лемана ПРО</t>
         </is>
       </c>
-      <c r="C10" s="51" t="inlineStr">
+      <c r="C10" s="60" t="inlineStr">
         <is>
           <t>В работах только подъём силами бригады</t>
         </is>
       </c>
-      <c r="D10" s="51" t="inlineStr">
+      <c r="D10" s="60" t="inlineStr">
         <is>
           <t>По тарифу магазина</t>
         </is>
       </c>
-      <c r="E10" s="51" t="inlineStr">
+      <c r="E10" s="60" t="inlineStr">
         <is>
           <t>Нет</t>
         </is>
       </c>
-      <c r="F10" s="57" t="inlineStr">
+      <c r="F10" s="66" t="inlineStr">
         <is>
           <t>НЕ ВХОДИТ</t>
         </is>
       </c>
     </row>
     <row r="11" ht="40" customHeight="1">
-      <c r="A11" s="50" t="n">
+      <c r="A11" s="59" t="n">
         <v>7</v>
       </c>
-      <c r="B11" s="51" t="inlineStr">
+      <c r="B11" s="60" t="inlineStr">
         <is>
           <t>Вывоз строительного мусора, контейнер</t>
         </is>
       </c>
-      <c r="C11" s="51" t="inlineStr">
-        <is>
-          <t>П. 10 работ — только уборка зоны, не вывоз</t>
-        </is>
-      </c>
-      <c r="D11" s="51" t="inlineStr">
+      <c r="C11" s="60" t="inlineStr">
+        <is>
+          <t>П. 9 работ на каждом балконе — только уборка зоны, не вывоз</t>
+        </is>
+      </c>
+      <c r="D11" s="60" t="inlineStr">
         <is>
           <t>Газель / контейнер отдельно</t>
         </is>
       </c>
-      <c r="E11" s="51" t="inlineStr">
+      <c r="E11" s="60" t="inlineStr">
         <is>
           <t>Нет</t>
         </is>
       </c>
-      <c r="F11" s="57" t="inlineStr">
+      <c r="F11" s="66" t="inlineStr">
         <is>
           <t>НЕ ВХОДИТ</t>
         </is>
       </c>
     </row>
     <row r="12" ht="40" customHeight="1">
-      <c r="A12" s="50" t="n">
+      <c r="A12" s="59" t="n">
         <v>8</v>
       </c>
-      <c r="B12" s="51" t="inlineStr">
+      <c r="B12" s="60" t="inlineStr">
         <is>
           <t>Наружная отделка ограждения, фасад, козырёк</t>
         </is>
       </c>
-      <c r="C12" s="51" t="inlineStr">
+      <c r="C12" s="60" t="inlineStr">
         <is>
           <t>Материалы только на внутренний контур</t>
         </is>
       </c>
-      <c r="D12" s="51" t="inlineStr">
+      <c r="D12" s="60" t="inlineStr">
         <is>
           <t>Отдельный вид работ</t>
         </is>
       </c>
-      <c r="E12" s="51" t="inlineStr">
+      <c r="E12" s="60" t="inlineStr">
         <is>
           <t>Да, если заказывать снаружи</t>
         </is>
       </c>
-      <c r="F12" s="57" t="inlineStr">
+      <c r="F12" s="66" t="inlineStr">
         <is>
           <t>НЕ ВХОДИТ</t>
         </is>
       </c>
     </row>
     <row r="13" ht="40" customHeight="1">
-      <c r="A13" s="50" t="n">
+      <c r="A13" s="59" t="n">
         <v>9</v>
       </c>
-      <c r="B13" s="51" t="inlineStr">
+      <c r="B13" s="60" t="inlineStr">
         <is>
           <t>Согласования, технадзор, скрытые работы</t>
         </is>
       </c>
-      <c r="C13" s="51" t="inlineStr">
+      <c r="C13" s="60" t="inlineStr">
         <is>
           <t>Не заказывались</t>
         </is>
       </c>
-      <c r="D13" s="51" t="inlineStr">
+      <c r="D13" s="60" t="inlineStr">
         <is>
           <t>По факту после вскрытия</t>
         </is>
       </c>
-      <c r="E13" s="51" t="inlineStr">
+      <c r="E13" s="60" t="inlineStr">
         <is>
           <t>Возможно</t>
         </is>
       </c>
-      <c r="F13" s="57" t="inlineStr">
+      <c r="F13" s="66" t="inlineStr">
         <is>
           <t>НЕ ВХОДИТ</t>
         </is>
       </c>
     </row>
     <row r="14" ht="40" customHeight="1">
-      <c r="A14" s="50" t="n">
+      <c r="A14" s="59" t="n">
         <v>10</v>
       </c>
-      <c r="B14" s="51" t="inlineStr">
+      <c r="B14" s="60" t="inlineStr">
         <is>
           <t>Покраска сверх 2 слоёв, колеровка, декоративка</t>
         </is>
       </c>
-      <c r="C14" s="51" t="inlineStr">
+      <c r="C14" s="60" t="inlineStr">
         <is>
           <t>В смете 2 слоя обычной краски</t>
         </is>
       </c>
-      <c r="D14" s="51" t="inlineStr">
+      <c r="D14" s="60" t="inlineStr">
         <is>
           <t>Доп. слой ~120–150 ₽/м²</t>
         </is>
       </c>
-      <c r="E14" s="51" t="inlineStr">
+      <c r="E14" s="60" t="inlineStr">
         <is>
           <t>Возможна доп. краска</t>
         </is>
       </c>
-      <c r="F14" s="57" t="inlineStr">
+      <c r="F14" s="66" t="inlineStr">
         <is>
           <t>НЕ ВХОДИТ</t>
         </is>
       </c>
     </row>
     <row r="15" ht="40" customHeight="1">
-      <c r="A15" s="50" t="n">
+      <c r="A15" s="59" t="n">
         <v>11</v>
       </c>
-      <c r="B15" s="51" t="inlineStr">
+      <c r="B15" s="60" t="inlineStr">
         <is>
           <t>Устройство порога / выход в комнату, демонтаж двери</t>
         </is>
       </c>
-      <c r="C15" s="51" t="inlineStr">
+      <c r="C15" s="60" t="inlineStr">
         <is>
           <t>В списке нет двери и порога</t>
         </is>
       </c>
-      <c r="D15" s="51" t="inlineStr">
+      <c r="D15" s="60" t="inlineStr">
         <is>
           <t>По месту</t>
         </is>
       </c>
-      <c r="E15" s="51" t="inlineStr">
+      <c r="E15" s="60" t="inlineStr">
         <is>
           <t>Да, если менять блок</t>
         </is>
       </c>
-      <c r="F15" s="57" t="inlineStr">
+      <c r="F15" s="66" t="inlineStr">
         <is>
           <t>НЕ ВХОДИТ</t>
         </is>
       </c>
     </row>
     <row r="16" ht="40" customHeight="1">
-      <c r="A16" s="50" t="n">
+      <c r="A16" s="59" t="n">
         <v>12</v>
       </c>
-      <c r="B16" s="51" t="inlineStr">
+      <c r="B16" s="60" t="inlineStr">
         <is>
           <t>Работа в ночь, срочность, простой из‑за погоды</t>
         </is>
       </c>
-      <c r="C16" s="51" t="inlineStr">
+      <c r="C16" s="60" t="inlineStr">
         <is>
           <t>Обычный дневной режим</t>
         </is>
       </c>
-      <c r="D16" s="51" t="inlineStr">
+      <c r="D16" s="60" t="inlineStr">
         <is>
           <t>Коэффициент 1,3–1,5</t>
         </is>
       </c>
-      <c r="E16" s="51" t="inlineStr">
+      <c r="E16" s="60" t="inlineStr">
         <is>
           <t>Нет</t>
         </is>
       </c>
-      <c r="F16" s="57" t="inlineStr">
+      <c r="F16" s="66" t="inlineStr">
         <is>
           <t>НЕ ВХОДИТ</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="58" t="inlineStr">
-        <is>
-          <t>Итог. В оплату по этой смете входят только работы со листа «Работы», строки 1–10, на сумму 23 395 ₽. Всё перечисленное выше в 23 395 ₽ не входит. Материалы оплачиваются отдельно (~20 708 ₽ по листу «Материалы»).</t>
-        </is>
-      </c>
-      <c r="B18" s="59" t="n"/>
-      <c r="C18" s="59" t="n"/>
-      <c r="D18" s="59" t="n"/>
-      <c r="E18" s="59" t="n"/>
-      <c r="F18" s="59" t="n"/>
+      <c r="A18" s="67" t="inlineStr">
+        <is>
+          <t>Итог. В оплату по этой смете входят только работы с листа «Работы»: 9 строк на каждый балкон, 22 495 ₽ × 2 = 44 990 ₽. Всё перечисленное выше в 44 990 ₽ не входит. Материалы оплачиваются отдельно (корзина Лемана ПРО / лист «Материалы»).</t>
+        </is>
+      </c>
+      <c r="B18" s="68" t="n"/>
+      <c r="C18" s="68" t="n"/>
+      <c r="D18" s="68" t="n"/>
+      <c r="E18" s="68" t="n"/>
+      <c r="F18" s="68" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="59" t="n"/>
-      <c r="B19" s="59" t="n"/>
-      <c r="C19" s="59" t="n"/>
-      <c r="D19" s="59" t="n"/>
-      <c r="E19" s="59" t="n"/>
-      <c r="F19" s="59" t="n"/>
+      <c r="A19" s="68" t="n"/>
+      <c r="B19" s="68" t="n"/>
+      <c r="C19" s="68" t="n"/>
+      <c r="D19" s="68" t="n"/>
+      <c r="E19" s="68" t="n"/>
+      <c r="F19" s="68" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="59" t="n"/>
-      <c r="B20" s="59" t="n"/>
-      <c r="C20" s="59" t="n"/>
-      <c r="D20" s="59" t="n"/>
-      <c r="E20" s="59" t="n"/>
-      <c r="F20" s="59" t="n"/>
+      <c r="A20" s="68" t="n"/>
+      <c r="B20" s="68" t="n"/>
+      <c r="C20" s="68" t="n"/>
+      <c r="D20" s="68" t="n"/>
+      <c r="E20" s="68" t="n"/>
+      <c r="F20" s="68" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -3477,7 +3885,7 @@
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="1" fitToWidth="1"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;LПервый балкон, Краснодар&amp;C13.10.2026&amp;R&amp;P из &amp;N</oddFooter>
+    <oddFooter>&amp;LДва балкона, Краснодар&amp;C13.10.2026&amp;R&amp;P из &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>

</xml_diff>